<commit_message>
To switch server and re-run optimization.
</commit_message>
<xml_diff>
--- a/temp/bad_2/optimization_results.xlsx
+++ b/temp/bad_2/optimization_results.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PinWei\AppData\Local\Temp\BvSshSftp-CM77XYMB\JLKTD499\R3PGAXWU\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PinWei\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2682A0FE-4366-4ACF-9A02-A55721738F38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F30BE5E3-AD74-4607-BBD3-DA4F84578888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-1524" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All Results" sheetId="1" r:id="rId1"/>
@@ -122,24 +122,25 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="12">
     <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
+          <bgColor theme="3" tint="0.749961851863155"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.749961851863155"/>
         </patternFill>
       </fill>
     </dxf>
@@ -150,16 +151,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -205,11 +196,41 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -8123,19 +8144,7 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G1:G1048576">
-    <cfRule type="colorScale" priority="6">
+    <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -8147,17 +8156,24 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1:F1048576">
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="6" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D1:D1048576">
-    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="0.09">
-      <formula>NOT(ISERROR(SEARCH("0.09",D1)))</formula>
+  <conditionalFormatting sqref="G1:G1048576">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:H1048576">
-    <cfRule type="colorScale" priority="1">
+    <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -8168,12 +8184,21 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="D1:D1048576">
+    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="inf">
+      <formula>NOT(ISERROR(SEARCH("inf",D1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="0.09">
+      <formula>NOT(ISERROR(SEARCH("0.09",D1)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{6B022D9B-699F-4EB9-A1C9-3C7C8C34C2A7}">
+          <x14:cfRule type="containsText" priority="5" operator="containsText" id="{6B022D9B-699F-4EB9-A1C9-3C7C8C34C2A7}">
             <xm:f>NOT(ISERROR(SEARCH(FALSE,E1)))</xm:f>
             <xm:f>FALSE</xm:f>
             <x14:dxf>

</xml_diff>